<commit_message>
Correcciones de la revisión: tipo de cambio BCE y aclaración del coste de Mistral (#6)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BPMkwzeUBA3i5SJoerRXPm
</commit_message>
<xml_diff>
--- a/docs/valores-reales-tickets.xlsx
+++ b/docs/valores-reales-tickets.xlsx
@@ -476,7 +476,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H31"/>
+  <dimension ref="A1:H39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -1356,7 +1356,7 @@
       </c>
       <c r="C28" s="6" t="inlineStr">
         <is>
-          <t>DUDOSO: NIF y número de factura poco nítidos. Base del 10 % leída como 44,58 (cuadra con el total 115,20). Total tras descuento de 1,58.</t>
+          <t>Revisado: NIF y número de factura comprobados. El número (132740032509026056) es coherente, según comprobó también Anaí: tienda 3274, fecha 25-09-02 y ticket 6056. Base del 10 % = 44,58 (cuadra con el total 115,20). Total tras descuento de 1,58.</t>
         </is>
       </c>
       <c r="D28" s="6" t="inlineStr">
@@ -1385,6 +1385,7 @@
         </is>
       </c>
     </row>
+    <row r="29"/>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
@@ -1399,6 +1400,14 @@
         </is>
       </c>
     </row>
+    <row r="32"/>
+    <row r="33"/>
+    <row r="34"/>
+    <row r="35"/>
+    <row r="36"/>
+    <row r="37"/>
+    <row r="38"/>
+    <row r="39"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Prueba de IA con el ticket real de gasolinera como T1 (#6)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BPMkwzeUBA3i5SJoerRXPm
</commit_message>
<xml_diff>
--- a/docs/valores-reales-tickets.xlsx
+++ b/docs/valores-reales-tickets.xlsx
@@ -476,7 +476,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H39"/>
+  <dimension ref="A1:I31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -487,6 +487,7 @@
     <col width="22" customWidth="1" min="6" max="6"/>
     <col width="22" customWidth="1" min="7" max="7"/>
     <col width="22" customWidth="1" min="8" max="8"/>
+    <col width="22" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -541,7 +542,7 @@
     <row r="8">
       <c r="A8" s="8" t="inlineStr">
         <is>
-          <t>Transcrito por Claude el 29/10/2026 a partir de las imágenes. Revisado y validado por Mireia el 29/10/2026.</t>
+          <t>Transcrito por Claude el 29/10/2026 y revisado por Mireia el mismo día. Columna T1 · Gasolinera añadida el 30/10/2026 con los valores de Ana (PR #48).</t>
         </is>
       </c>
     </row>
@@ -553,35 +554,40 @@
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>T1 · Alcampo arrugado</t>
+          <t>T1 · Gasolinera arrugado</t>
         </is>
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
+          <t>E4 · Alcampo arrugado (antes sustituto de T1)</t>
+        </is>
+      </c>
+      <c r="D9" s="4" t="inlineStr">
+        <is>
           <t>T2 · Eroski varios IVA</t>
         </is>
       </c>
-      <c r="D9" s="4" t="inlineStr">
+      <c r="E9" s="4" t="inlineStr">
         <is>
           <t>T3 · Claude Pro (inglés)</t>
         </is>
       </c>
-      <c r="E9" s="4" t="inlineStr">
+      <c r="F9" s="4" t="inlineStr">
         <is>
           <t>T4 · Cervecería poca luz</t>
         </is>
       </c>
-      <c r="F9" s="4" t="inlineStr">
+      <c r="G9" s="4" t="inlineStr">
         <is>
           <t>E1 · AUCALSA peaje</t>
         </is>
       </c>
-      <c r="G9" s="4" t="inlineStr">
+      <c r="H9" s="4" t="inlineStr">
         <is>
           <t>E2 · Carrefour (PDF)</t>
         </is>
       </c>
-      <c r="H9" s="4" t="inlineStr">
+      <c r="I9" s="4" t="inlineStr">
         <is>
           <t>E3 · Druni (PDF)</t>
         </is>
@@ -595,35 +601,40 @@
       </c>
       <c r="B10" s="6" t="inlineStr">
         <is>
+          <t>2026-03-07</t>
+        </is>
+      </c>
+      <c r="C10" s="6" t="inlineStr">
+        <is>
           <t>2026-09-08</t>
         </is>
       </c>
-      <c r="C10" s="6" t="inlineStr">
+      <c r="D10" s="6" t="inlineStr">
         <is>
           <t>2025-09-02</t>
         </is>
       </c>
-      <c r="D10" s="6" t="inlineStr">
+      <c r="E10" s="6" t="inlineStr">
         <is>
           <t>2026-10-14</t>
         </is>
       </c>
-      <c r="E10" s="6" t="inlineStr">
+      <c r="F10" s="6" t="inlineStr">
         <is>
           <t>2026-08-29</t>
         </is>
       </c>
-      <c r="F10" s="6" t="inlineStr">
+      <c r="G10" s="6" t="inlineStr">
         <is>
           <t>2026-10-25</t>
         </is>
       </c>
-      <c r="G10" s="6" t="inlineStr">
+      <c r="H10" s="6" t="inlineStr">
         <is>
           <t>2026-10-19</t>
         </is>
       </c>
-      <c r="H10" s="6" t="inlineStr">
+      <c r="I10" s="6" t="inlineStr">
         <is>
           <t>2026-06-25</t>
         </is>
@@ -637,35 +648,40 @@
       </c>
       <c r="B11" s="6" t="inlineStr">
         <is>
+          <t>E.S. Villaquejida - Sutecal</t>
+        </is>
+      </c>
+      <c r="C11" s="6" t="inlineStr">
+        <is>
           <t>Alcampo Santa Nonia</t>
         </is>
       </c>
-      <c r="C11" s="6" t="inlineStr">
+      <c r="D11" s="6" t="inlineStr">
         <is>
           <t>Vego Supermercados S.A.U.</t>
         </is>
       </c>
-      <c r="D11" s="6" t="inlineStr">
+      <c r="E11" s="6" t="inlineStr">
         <is>
           <t>Anthropic Ireland, Limited</t>
         </is>
       </c>
-      <c r="E11" s="6" t="inlineStr">
+      <c r="F11" s="6" t="inlineStr">
         <is>
           <t>Cerveceria Celtica S.L.</t>
         </is>
       </c>
-      <c r="F11" s="6" t="inlineStr">
+      <c r="G11" s="6" t="inlineStr">
         <is>
           <t>AUCALSA</t>
         </is>
       </c>
-      <c r="G11" s="6" t="inlineStr">
+      <c r="H11" s="6" t="inlineStr">
         <is>
           <t>Centros Comerciales Carrefour S.A.</t>
         </is>
       </c>
-      <c r="H11" s="6" t="inlineStr">
+      <c r="I11" s="6" t="inlineStr">
         <is>
           <t>DRUNI, S.A.</t>
         </is>
@@ -679,35 +695,40 @@
       </c>
       <c r="B12" s="6" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>B49268071</t>
         </is>
       </c>
       <c r="C12" s="6" t="inlineStr">
         <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="D12" s="6" t="inlineStr">
+        <is>
           <t>A36651313</t>
         </is>
       </c>
-      <c r="D12" s="6" t="inlineStr">
+      <c r="E12" s="6" t="inlineStr">
         <is>
           <t>IE4276970QH</t>
         </is>
       </c>
-      <c r="E12" s="6" t="inlineStr">
+      <c r="F12" s="6" t="inlineStr">
         <is>
           <t>B24610297</t>
         </is>
       </c>
-      <c r="F12" s="6" t="inlineStr">
+      <c r="G12" s="6" t="inlineStr">
         <is>
           <t>A28415784</t>
         </is>
       </c>
-      <c r="G12" s="6" t="inlineStr">
+      <c r="H12" s="6" t="inlineStr">
         <is>
           <t>A28425270</t>
         </is>
       </c>
-      <c r="H12" s="6" t="inlineStr">
+      <c r="I12" s="6" t="inlineStr">
         <is>
           <t>A46581666</t>
         </is>
@@ -754,6 +775,11 @@
           <t>N/A</t>
         </is>
       </c>
+      <c r="I13" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="5" t="inlineStr">
@@ -763,35 +789,40 @@
       </c>
       <c r="B14" s="6" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>2023018651</t>
         </is>
       </c>
       <c r="C14" s="6" t="inlineStr">
         <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="D14" s="6" t="inlineStr">
+        <is>
           <t>132740032509026056</t>
         </is>
       </c>
-      <c r="D14" s="6" t="inlineStr">
+      <c r="E14" s="6" t="inlineStr">
         <is>
           <t>9BF0758D-8771996</t>
         </is>
       </c>
-      <c r="E14" s="6" t="inlineStr">
+      <c r="F14" s="6" t="inlineStr">
         <is>
           <t>1 / 388087</t>
         </is>
       </c>
-      <c r="F14" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
       <c r="G14" s="6" t="inlineStr">
         <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H14" s="6" t="inlineStr">
+        <is>
           <t>N0020008261019000107</t>
         </is>
       </c>
-      <c r="H14" s="6" t="inlineStr">
+      <c r="I14" s="6" t="inlineStr">
         <is>
           <t>20832606010734</t>
         </is>
@@ -805,35 +836,40 @@
       </c>
       <c r="B15" s="6" t="inlineStr">
         <is>
+          <t>21</t>
+        </is>
+      </c>
+      <c r="C15" s="6" t="inlineStr">
+        <is>
           <t>4</t>
         </is>
       </c>
-      <c r="C15" s="6" t="inlineStr">
+      <c r="D15" s="6" t="inlineStr">
         <is>
           <t>10</t>
         </is>
       </c>
-      <c r="D15" s="6" t="inlineStr">
+      <c r="E15" s="6" t="inlineStr">
         <is>
           <t>21</t>
         </is>
       </c>
-      <c r="E15" s="6" t="inlineStr">
+      <c r="F15" s="6" t="inlineStr">
         <is>
           <t>10</t>
         </is>
       </c>
-      <c r="F15" s="6" t="inlineStr">
+      <c r="G15" s="6" t="inlineStr">
         <is>
           <t>21</t>
         </is>
       </c>
-      <c r="G15" s="6" t="inlineStr">
+      <c r="H15" s="6" t="inlineStr">
         <is>
           <t>21</t>
         </is>
       </c>
-      <c r="H15" s="6" t="inlineStr">
+      <c r="I15" s="6" t="inlineStr">
         <is>
           <t>21</t>
         </is>
@@ -847,35 +883,40 @@
       </c>
       <c r="B16" s="6" t="inlineStr">
         <is>
+          <t>88,21</t>
+        </is>
+      </c>
+      <c r="C16" s="6" t="inlineStr">
+        <is>
           <t>4,05</t>
         </is>
       </c>
-      <c r="C16" s="6" t="inlineStr">
+      <c r="D16" s="6" t="inlineStr">
         <is>
           <t>44,58</t>
         </is>
       </c>
-      <c r="D16" s="6" t="inlineStr">
+      <c r="E16" s="6" t="inlineStr">
         <is>
           <t>18,00</t>
         </is>
       </c>
-      <c r="E16" s="6" t="inlineStr">
+      <c r="F16" s="6" t="inlineStr">
         <is>
           <t>19,09</t>
         </is>
       </c>
-      <c r="F16" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
       <c r="G16" s="6" t="inlineStr">
         <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H16" s="6" t="inlineStr">
+        <is>
           <t>8,26</t>
         </is>
       </c>
-      <c r="H16" s="6" t="inlineStr">
+      <c r="I16" s="6" t="inlineStr">
         <is>
           <t>17,28</t>
         </is>
@@ -889,35 +930,40 @@
       </c>
       <c r="B17" s="6" t="inlineStr">
         <is>
+          <t>18,53</t>
+        </is>
+      </c>
+      <c r="C17" s="6" t="inlineStr">
+        <is>
           <t>0,15</t>
         </is>
       </c>
-      <c r="C17" s="6" t="inlineStr">
+      <c r="D17" s="6" t="inlineStr">
         <is>
           <t>4,46</t>
         </is>
       </c>
-      <c r="D17" s="6" t="inlineStr">
+      <c r="E17" s="6" t="inlineStr">
         <is>
           <t>3,78</t>
         </is>
       </c>
-      <c r="E17" s="6" t="inlineStr">
+      <c r="F17" s="6" t="inlineStr">
         <is>
           <t>1,91</t>
         </is>
       </c>
-      <c r="F17" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
       <c r="G17" s="6" t="inlineStr">
         <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H17" s="6" t="inlineStr">
+        <is>
           <t>1,73</t>
         </is>
       </c>
-      <c r="H17" s="6" t="inlineStr">
+      <c r="I17" s="6" t="inlineStr">
         <is>
           <t>3,63</t>
         </is>
@@ -931,19 +977,19 @@
       </c>
       <c r="B18" s="6" t="inlineStr">
         <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="C18" s="6" t="inlineStr">
+        <is>
           <t>21</t>
         </is>
       </c>
-      <c r="C18" s="6" t="inlineStr">
+      <c r="D18" s="6" t="inlineStr">
         <is>
           <t>21</t>
         </is>
       </c>
-      <c r="D18" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
       <c r="E18" s="6" t="inlineStr">
         <is>
           <t>N/A</t>
@@ -960,6 +1006,11 @@
         </is>
       </c>
       <c r="H18" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="I18" s="6" t="inlineStr">
         <is>
           <t>4</t>
         </is>
@@ -973,19 +1024,19 @@
       </c>
       <c r="B19" s="6" t="inlineStr">
         <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="C19" s="6" t="inlineStr">
+        <is>
           <t>1,31</t>
         </is>
       </c>
-      <c r="C19" s="6" t="inlineStr">
+      <c r="D19" s="6" t="inlineStr">
         <is>
           <t>10,29</t>
         </is>
       </c>
-      <c r="D19" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
       <c r="E19" s="6" t="inlineStr">
         <is>
           <t>N/A</t>
@@ -1002,6 +1053,11 @@
         </is>
       </c>
       <c r="H19" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="I19" s="6" t="inlineStr">
         <is>
           <t>7,67</t>
         </is>
@@ -1015,19 +1071,19 @@
       </c>
       <c r="B20" s="6" t="inlineStr">
         <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="C20" s="6" t="inlineStr">
+        <is>
           <t>0,28</t>
         </is>
       </c>
-      <c r="C20" s="6" t="inlineStr">
+      <c r="D20" s="6" t="inlineStr">
         <is>
           <t>2,16</t>
         </is>
       </c>
-      <c r="D20" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
       <c r="E20" s="6" t="inlineStr">
         <is>
           <t>N/A</t>
@@ -1044,6 +1100,11 @@
         </is>
       </c>
       <c r="H20" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="I20" s="6" t="inlineStr">
         <is>
           <t>0,31</t>
         </is>
@@ -1062,14 +1123,14 @@
       </c>
       <c r="C21" s="6" t="inlineStr">
         <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="D21" s="6" t="inlineStr">
+        <is>
           <t>4</t>
         </is>
       </c>
-      <c r="D21" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
       <c r="E21" s="6" t="inlineStr">
         <is>
           <t>N/A</t>
@@ -1086,6 +1147,11 @@
         </is>
       </c>
       <c r="H21" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="I21" s="6" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
@@ -1104,14 +1170,14 @@
       </c>
       <c r="C22" s="6" t="inlineStr">
         <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="D22" s="6" t="inlineStr">
+        <is>
           <t>51,64</t>
         </is>
       </c>
-      <c r="D22" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
       <c r="E22" s="6" t="inlineStr">
         <is>
           <t>N/A</t>
@@ -1128,6 +1194,11 @@
         </is>
       </c>
       <c r="H22" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="I22" s="6" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
@@ -1146,14 +1217,14 @@
       </c>
       <c r="C23" s="6" t="inlineStr">
         <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="D23" s="6" t="inlineStr">
+        <is>
           <t>2,07</t>
         </is>
       </c>
-      <c r="D23" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
       <c r="E23" s="6" t="inlineStr">
         <is>
           <t>N/A</t>
@@ -1170,6 +1241,11 @@
         </is>
       </c>
       <c r="H23" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="I23" s="6" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
@@ -1183,35 +1259,40 @@
       </c>
       <c r="B24" s="6" t="inlineStr">
         <is>
+          <t>88,21</t>
+        </is>
+      </c>
+      <c r="C24" s="6" t="inlineStr">
+        <is>
           <t>5,36</t>
         </is>
       </c>
-      <c r="C24" s="6" t="inlineStr">
+      <c r="D24" s="6" t="inlineStr">
         <is>
           <t>106,51</t>
         </is>
       </c>
-      <c r="D24" s="6" t="inlineStr">
+      <c r="E24" s="6" t="inlineStr">
         <is>
           <t>18,00</t>
         </is>
       </c>
-      <c r="E24" s="6" t="inlineStr">
+      <c r="F24" s="6" t="inlineStr">
         <is>
           <t>19,09</t>
         </is>
       </c>
-      <c r="F24" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
       <c r="G24" s="6" t="inlineStr">
         <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H24" s="6" t="inlineStr">
+        <is>
           <t>8,26</t>
         </is>
       </c>
-      <c r="H24" s="6" t="inlineStr">
+      <c r="I24" s="6" t="inlineStr">
         <is>
           <t>24,95</t>
         </is>
@@ -1225,35 +1306,40 @@
       </c>
       <c r="B25" s="6" t="inlineStr">
         <is>
+          <t>106,74</t>
+        </is>
+      </c>
+      <c r="C25" s="6" t="inlineStr">
+        <is>
           <t>5,79</t>
         </is>
       </c>
-      <c r="C25" s="6" t="inlineStr">
+      <c r="D25" s="6" t="inlineStr">
         <is>
           <t>115,20</t>
         </is>
       </c>
-      <c r="D25" s="6" t="inlineStr">
+      <c r="E25" s="6" t="inlineStr">
         <is>
           <t>21,78</t>
         </is>
       </c>
-      <c r="E25" s="6" t="inlineStr">
+      <c r="F25" s="6" t="inlineStr">
         <is>
           <t>21,00</t>
         </is>
       </c>
-      <c r="F25" s="6" t="inlineStr">
+      <c r="G25" s="6" t="inlineStr">
         <is>
           <t>10,20</t>
         </is>
       </c>
-      <c r="G25" s="6" t="inlineStr">
+      <c r="H25" s="6" t="inlineStr">
         <is>
           <t>9,99</t>
         </is>
       </c>
-      <c r="H25" s="6" t="inlineStr">
+      <c r="I25" s="6" t="inlineStr">
         <is>
           <t>28,89</t>
         </is>
@@ -1300,6 +1386,11 @@
           <t>EUR</t>
         </is>
       </c>
+      <c r="I26" s="6" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="5" t="inlineStr">
@@ -1309,35 +1400,40 @@
       </c>
       <c r="B27" s="6" t="inlineStr">
         <is>
+          <t>Combustible y transporte</t>
+        </is>
+      </c>
+      <c r="C27" s="6" t="inlineStr">
+        <is>
           <t>Alimentación</t>
         </is>
       </c>
-      <c r="C27" s="6" t="inlineStr">
+      <c r="D27" s="6" t="inlineStr">
         <is>
           <t>Alimentación</t>
         </is>
       </c>
-      <c r="D27" s="6" t="inlineStr">
+      <c r="E27" s="6" t="inlineStr">
         <is>
           <t>Software y suscripciones</t>
         </is>
       </c>
-      <c r="E27" s="6" t="inlineStr">
+      <c r="F27" s="6" t="inlineStr">
         <is>
           <t>Restauración y dietas</t>
         </is>
       </c>
-      <c r="F27" s="6" t="inlineStr">
+      <c r="G27" s="6" t="inlineStr">
         <is>
           <t>Combustible y transporte</t>
         </is>
       </c>
-      <c r="G27" s="6" t="inlineStr">
+      <c r="H27" s="6" t="inlineStr">
         <is>
           <t>Otros</t>
         </is>
       </c>
-      <c r="H27" s="6" t="inlineStr">
+      <c r="I27" s="6" t="inlineStr">
         <is>
           <t>Otros</t>
         </is>
@@ -1351,35 +1447,40 @@
       </c>
       <c r="B28" s="6" t="inlineStr">
         <is>
+          <t>Valores aportados por Ana en el PR #48 y comprobados: 88,21 + 18,53 = 106,74 € y 59,40 L × 1,797 = 106,74 €.</t>
+        </is>
+      </c>
+      <c r="C28" s="6" t="inlineStr">
+        <is>
           <t>No se ve NIF del emisor ni número de factura en la foto (puede estar en la parte cortada). Cuota del 4 % impresa ,15 (4,05+0,15 = 4,20 = 3 panes).</t>
         </is>
       </c>
-      <c r="C28" s="6" t="inlineStr">
+      <c r="D28" s="6" t="inlineStr">
         <is>
           <t>Revisado: NIF y número de factura comprobados. El número (132740032509026056) es coherente, según comprobó también Anaí: tienda 3274, fecha 25-09-02 y ticket 6056. Base del 10 % = 44,58 (cuadra con el total 115,20). Total tras descuento de 1,58.</t>
         </is>
       </c>
-      <c r="D28" s="6" t="inlineStr">
+      <c r="E28" s="6" t="inlineStr">
         <is>
           <t>El receptor es particular, sin NIF. Nombre del receptor tapado.</t>
         </is>
       </c>
-      <c r="E28" s="6" t="inlineStr">
+      <c r="F28" s="6" t="inlineStr">
         <is>
           <t>El dedo tapa parte de 'TOTAL EUROS', pero el importe 21,00 se ve.</t>
         </is>
       </c>
-      <c r="F28" s="6" t="inlineStr">
+      <c r="G28" s="6" t="inlineStr">
         <is>
           <t>Ticket de peaje, no factura. Solo pone 'IVA 21 % incluido': calculado, base 8,43 y cuota 1,77. Sin número de factura (N. tránsito 69245-0096).</t>
         </is>
       </c>
-      <c r="G28" s="6" t="inlineStr">
+      <c r="H28" s="6" t="inlineStr">
         <is>
           <t>Número tomado del 'NRF'. Champú: categoría 'Otros' (no hay categoría de higiene).</t>
         </is>
       </c>
-      <c r="H28" s="6" t="inlineStr">
+      <c r="I28" s="6" t="inlineStr">
         <is>
           <t>Perfumería: categoría 'Otros'.</t>
         </is>
@@ -1400,14 +1501,6 @@
         </is>
       </c>
     </row>
-    <row r="32"/>
-    <row r="33"/>
-    <row r="34"/>
-    <row r="35"/>
-    <row r="36"/>
-    <row r="37"/>
-    <row r="38"/>
-    <row r="39"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Prueba de IA con la foto torcida y con poca luz (T4b) (#6)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BPMkwzeUBA3i5SJoerRXPm
</commit_message>
<xml_diff>
--- a/docs/valores-reales-tickets.xlsx
+++ b/docs/valores-reales-tickets.xlsx
@@ -476,7 +476,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I31"/>
+  <dimension ref="A1:J31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -488,6 +488,7 @@
     <col width="22" customWidth="1" min="7" max="7"/>
     <col width="22" customWidth="1" min="8" max="8"/>
     <col width="22" customWidth="1" min="9" max="9"/>
+    <col width="22" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -542,7 +543,7 @@
     <row r="8">
       <c r="A8" s="8" t="inlineStr">
         <is>
-          <t>Transcrito por Claude el 29/10/2026 y revisado por Mireia el mismo día. Columna T1 · Gasolinera añadida el 30/10/2026 con los valores de Ana (PR #48).</t>
+          <t>Transcrito por Claude el 29/10/2026 y revisado por Mireia el mismo día. Columna T1 · Gasolinera añadida el 30/10/2026 con los valores de Ana (PR #48). Columna T4b añadida el 30/10/2026 con los valores de Ana (PR #59).</t>
         </is>
       </c>
     </row>
@@ -579,15 +580,20 @@
       </c>
       <c r="G9" s="4" t="inlineStr">
         <is>
+          <t>T4b · Mercadona torcida y poca luz</t>
+        </is>
+      </c>
+      <c r="H9" s="4" t="inlineStr">
+        <is>
           <t>E1 · AUCALSA peaje</t>
         </is>
       </c>
-      <c r="H9" s="4" t="inlineStr">
+      <c r="I9" s="4" t="inlineStr">
         <is>
           <t>E2 · Carrefour (PDF)</t>
         </is>
       </c>
-      <c r="I9" s="4" t="inlineStr">
+      <c r="J9" s="4" t="inlineStr">
         <is>
           <t>E3 · Druni (PDF)</t>
         </is>
@@ -626,15 +632,20 @@
       </c>
       <c r="G10" s="6" t="inlineStr">
         <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="H10" s="6" t="inlineStr">
+        <is>
           <t>2026-10-25</t>
         </is>
       </c>
-      <c r="H10" s="6" t="inlineStr">
+      <c r="I10" s="6" t="inlineStr">
         <is>
           <t>2026-10-19</t>
         </is>
       </c>
-      <c r="I10" s="6" t="inlineStr">
+      <c r="J10" s="6" t="inlineStr">
         <is>
           <t>2026-06-25</t>
         </is>
@@ -673,15 +684,20 @@
       </c>
       <c r="G11" s="6" t="inlineStr">
         <is>
+          <t>Mercadona, S.A.</t>
+        </is>
+      </c>
+      <c r="H11" s="6" t="inlineStr">
+        <is>
           <t>AUCALSA</t>
         </is>
       </c>
-      <c r="H11" s="6" t="inlineStr">
+      <c r="I11" s="6" t="inlineStr">
         <is>
           <t>Centros Comerciales Carrefour S.A.</t>
         </is>
       </c>
-      <c r="I11" s="6" t="inlineStr">
+      <c r="J11" s="6" t="inlineStr">
         <is>
           <t>DRUNI, S.A.</t>
         </is>
@@ -720,15 +736,20 @@
       </c>
       <c r="G12" s="6" t="inlineStr">
         <is>
+          <t>A46103834</t>
+        </is>
+      </c>
+      <c r="H12" s="6" t="inlineStr">
+        <is>
           <t>A28415784</t>
         </is>
       </c>
-      <c r="H12" s="6" t="inlineStr">
+      <c r="I12" s="6" t="inlineStr">
         <is>
           <t>A28425270</t>
         </is>
       </c>
-      <c r="I12" s="6" t="inlineStr">
+      <c r="J12" s="6" t="inlineStr">
         <is>
           <t>A46581666</t>
         </is>
@@ -780,6 +801,11 @@
           <t>N/A</t>
         </is>
       </c>
+      <c r="J13" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="5" t="inlineStr">
@@ -814,15 +840,20 @@
       </c>
       <c r="G14" s="6" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>2939-017-128100</t>
         </is>
       </c>
       <c r="H14" s="6" t="inlineStr">
         <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="I14" s="6" t="inlineStr">
+        <is>
           <t>N0020008261019000107</t>
         </is>
       </c>
-      <c r="I14" s="6" t="inlineStr">
+      <c r="J14" s="6" t="inlineStr">
         <is>
           <t>20832606010734</t>
         </is>
@@ -861,15 +892,20 @@
       </c>
       <c r="G15" s="6" t="inlineStr">
         <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="H15" s="6" t="inlineStr">
+        <is>
           <t>21</t>
         </is>
       </c>
-      <c r="H15" s="6" t="inlineStr">
+      <c r="I15" s="6" t="inlineStr">
         <is>
           <t>21</t>
         </is>
       </c>
-      <c r="I15" s="6" t="inlineStr">
+      <c r="J15" s="6" t="inlineStr">
         <is>
           <t>21</t>
         </is>
@@ -908,15 +944,20 @@
       </c>
       <c r="G16" s="6" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>10,66</t>
         </is>
       </c>
       <c r="H16" s="6" t="inlineStr">
         <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="I16" s="6" t="inlineStr">
+        <is>
           <t>8,26</t>
         </is>
       </c>
-      <c r="I16" s="6" t="inlineStr">
+      <c r="J16" s="6" t="inlineStr">
         <is>
           <t>17,28</t>
         </is>
@@ -955,15 +996,20 @@
       </c>
       <c r="G17" s="6" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>0,43</t>
         </is>
       </c>
       <c r="H17" s="6" t="inlineStr">
         <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="I17" s="6" t="inlineStr">
+        <is>
           <t>1,73</t>
         </is>
       </c>
-      <c r="I17" s="6" t="inlineStr">
+      <c r="J17" s="6" t="inlineStr">
         <is>
           <t>3,63</t>
         </is>
@@ -1002,7 +1048,7 @@
       </c>
       <c r="G18" s="6" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>10</t>
         </is>
       </c>
       <c r="H18" s="6" t="inlineStr">
@@ -1011,6 +1057,11 @@
         </is>
       </c>
       <c r="I18" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="J18" s="6" t="inlineStr">
         <is>
           <t>4</t>
         </is>
@@ -1049,7 +1100,7 @@
       </c>
       <c r="G19" s="6" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>29,95</t>
         </is>
       </c>
       <c r="H19" s="6" t="inlineStr">
@@ -1058,6 +1109,11 @@
         </is>
       </c>
       <c r="I19" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="J19" s="6" t="inlineStr">
         <is>
           <t>7,67</t>
         </is>
@@ -1096,7 +1152,7 @@
       </c>
       <c r="G20" s="6" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>2,99</t>
         </is>
       </c>
       <c r="H20" s="6" t="inlineStr">
@@ -1105,6 +1161,11 @@
         </is>
       </c>
       <c r="I20" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="J20" s="6" t="inlineStr">
         <is>
           <t>0,31</t>
         </is>
@@ -1143,7 +1204,7 @@
       </c>
       <c r="G21" s="6" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>21</t>
         </is>
       </c>
       <c r="H21" s="6" t="inlineStr">
@@ -1152,6 +1213,11 @@
         </is>
       </c>
       <c r="I21" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="J21" s="6" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
@@ -1190,7 +1256,7 @@
       </c>
       <c r="G22" s="6" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>10,33</t>
         </is>
       </c>
       <c r="H22" s="6" t="inlineStr">
@@ -1199,6 +1265,11 @@
         </is>
       </c>
       <c r="I22" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="J22" s="6" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
@@ -1237,7 +1308,7 @@
       </c>
       <c r="G23" s="6" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>2,17</t>
         </is>
       </c>
       <c r="H23" s="6" t="inlineStr">
@@ -1246,6 +1317,11 @@
         </is>
       </c>
       <c r="I23" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="J23" s="6" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
@@ -1284,15 +1360,20 @@
       </c>
       <c r="G24" s="6" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>50,94</t>
         </is>
       </c>
       <c r="H24" s="6" t="inlineStr">
         <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="I24" s="6" t="inlineStr">
+        <is>
           <t>8,26</t>
         </is>
       </c>
-      <c r="I24" s="6" t="inlineStr">
+      <c r="J24" s="6" t="inlineStr">
         <is>
           <t>24,95</t>
         </is>
@@ -1331,15 +1412,20 @@
       </c>
       <c r="G25" s="6" t="inlineStr">
         <is>
+          <t>56,53</t>
+        </is>
+      </c>
+      <c r="H25" s="6" t="inlineStr">
+        <is>
           <t>10,20</t>
         </is>
       </c>
-      <c r="H25" s="6" t="inlineStr">
+      <c r="I25" s="6" t="inlineStr">
         <is>
           <t>9,99</t>
         </is>
       </c>
-      <c r="I25" s="6" t="inlineStr">
+      <c r="J25" s="6" t="inlineStr">
         <is>
           <t>28,89</t>
         </is>
@@ -1391,6 +1477,11 @@
           <t>EUR</t>
         </is>
       </c>
+      <c r="J26" s="6" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="5" t="inlineStr">
@@ -1425,15 +1516,20 @@
       </c>
       <c r="G27" s="6" t="inlineStr">
         <is>
+          <t>Alimentación</t>
+        </is>
+      </c>
+      <c r="H27" s="6" t="inlineStr">
+        <is>
           <t>Combustible y transporte</t>
         </is>
       </c>
-      <c r="H27" s="6" t="inlineStr">
+      <c r="I27" s="6" t="inlineStr">
         <is>
           <t>Otros</t>
         </is>
       </c>
-      <c r="I27" s="6" t="inlineStr">
+      <c r="J27" s="6" t="inlineStr">
         <is>
           <t>Otros</t>
         </is>
@@ -1472,15 +1568,20 @@
       </c>
       <c r="G28" s="6" t="inlineStr">
         <is>
+          <t>Valores del PR #59; número de factura confirmado por Ana con el ticket en papel. Trampa: la foto lleva la fecha de la cámara (30/10/2026).</t>
+        </is>
+      </c>
+      <c r="H28" s="6" t="inlineStr">
+        <is>
           <t>Ticket de peaje, no factura. Solo pone 'IVA 21 % incluido': calculado, base 8,43 y cuota 1,77. Sin número de factura (N. tránsito 69245-0096).</t>
         </is>
       </c>
-      <c r="H28" s="6" t="inlineStr">
+      <c r="I28" s="6" t="inlineStr">
         <is>
           <t>Número tomado del 'NRF'. Champú: categoría 'Otros' (no hay categoría de higiene).</t>
         </is>
       </c>
-      <c r="I28" s="6" t="inlineStr">
+      <c r="J28" s="6" t="inlineStr">
         <is>
           <t>Perfumería: categoría 'Otros'.</t>
         </is>

</xml_diff>

<commit_message>
Prueba de IA con el ticket en pesos mexicanos (E5) (#6)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BPMkwzeUBA3i5SJoerRXPm
</commit_message>
<xml_diff>
--- a/docs/valores-reales-tickets.xlsx
+++ b/docs/valores-reales-tickets.xlsx
@@ -476,7 +476,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J31"/>
+  <dimension ref="A1:K31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -489,6 +489,7 @@
     <col width="22" customWidth="1" min="8" max="8"/>
     <col width="22" customWidth="1" min="9" max="9"/>
     <col width="22" customWidth="1" min="10" max="10"/>
+    <col width="24" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -543,7 +544,7 @@
     <row r="8">
       <c r="A8" s="8" t="inlineStr">
         <is>
-          <t>Transcrito por Claude el 29/10/2026 y revisado por Mireia el mismo día. Columna T1 · Gasolinera añadida el 30/10/2026 con los valores de Ana (PR #48). Columna T4b añadida el 30/10/2026 con los valores de Ana (PR #59).</t>
+          <t>Transcrito por Claude el 29/10/2026 y revisado por Mireia el mismo día. Columna T1 · Gasolinera añadida el 30/10/2026 con los valores de Ana (PR #48). Columna T4b añadida el 30/10/2026 con los valores de Ana (PR #59). Columna E5 añadida el 30/10/2026 con los valores de Ana (PR #62).</t>
         </is>
       </c>
     </row>
@@ -598,6 +599,11 @@
           <t>E3 · Druni (PDF)</t>
         </is>
       </c>
+      <c r="K9" s="4" t="inlineStr">
+        <is>
+          <t>E5 · Bodega Aurrera (pesos mexicanos)</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
@@ -650,6 +656,11 @@
           <t>2026-06-25</t>
         </is>
       </c>
+      <c r="K10" s="6" t="inlineStr">
+        <is>
+          <t>2024-01-06</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="5" t="inlineStr">
@@ -702,6 +713,11 @@
           <t>DRUNI, S.A.</t>
         </is>
       </c>
+      <c r="K11" s="6" t="inlineStr">
+        <is>
+          <t>Nueva Wal Mart de México S. de R.L. de C.V. (Bodega Aurrera)</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
@@ -754,6 +770,11 @@
           <t>A46581666</t>
         </is>
       </c>
+      <c r="K12" s="6" t="inlineStr">
+        <is>
+          <t>NWM9709244W4 (RFC)</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="5" t="inlineStr">
@@ -806,6 +827,11 @@
           <t>N/A</t>
         </is>
       </c>
+      <c r="K13" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="5" t="inlineStr">
@@ -858,6 +884,11 @@
           <t>20832606010734</t>
         </is>
       </c>
+      <c r="K14" s="6" t="inlineStr">
+        <is>
+          <t>01976 (TR#)</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="5" t="inlineStr">
@@ -910,6 +941,11 @@
           <t>21</t>
         </is>
       </c>
+      <c r="K15" s="6" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="5" t="inlineStr">
@@ -962,6 +998,11 @@
           <t>17,28</t>
         </is>
       </c>
+      <c r="K16" s="6" t="inlineStr">
+        <is>
+          <t>323,62</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="5" t="inlineStr">
@@ -1014,6 +1055,11 @@
           <t>3,63</t>
         </is>
       </c>
+      <c r="K17" s="6" t="inlineStr">
+        <is>
+          <t>25,89</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="5" t="inlineStr">
@@ -1066,6 +1112,11 @@
           <t>4</t>
         </is>
       </c>
+      <c r="K18" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="5" t="inlineStr">
@@ -1118,6 +1169,11 @@
           <t>7,67</t>
         </is>
       </c>
+      <c r="K19" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="5" t="inlineStr">
@@ -1170,6 +1226,11 @@
           <t>0,31</t>
         </is>
       </c>
+      <c r="K20" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="5" t="inlineStr">
@@ -1222,6 +1283,11 @@
           <t>N/A</t>
         </is>
       </c>
+      <c r="K21" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="5" t="inlineStr">
@@ -1274,6 +1340,11 @@
           <t>N/A</t>
         </is>
       </c>
+      <c r="K22" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="5" t="inlineStr">
@@ -1326,6 +1397,11 @@
           <t>N/A</t>
         </is>
       </c>
+      <c r="K23" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="5" t="inlineStr">
@@ -1378,6 +1454,11 @@
           <t>24,95</t>
         </is>
       </c>
+      <c r="K24" s="6" t="inlineStr">
+        <is>
+          <t>323,62</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="5" t="inlineStr">
@@ -1430,6 +1511,11 @@
           <t>28,89</t>
         </is>
       </c>
+      <c r="K25" s="6" t="inlineStr">
+        <is>
+          <t>635,02</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="5" t="inlineStr">
@@ -1482,6 +1568,11 @@
           <t>EUR</t>
         </is>
       </c>
+      <c r="K26" s="6" t="inlineStr">
+        <is>
+          <t>MXN</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="5" t="inlineStr">
@@ -1534,6 +1625,11 @@
           <t>Otros</t>
         </is>
       </c>
+      <c r="K27" s="6" t="inlineStr">
+        <is>
+          <t>Alimentación</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="5" t="inlineStr">
@@ -1586,8 +1682,12 @@
           <t>Perfumería: categoría 'Otros'.</t>
         </is>
       </c>
-    </row>
-    <row r="29"/>
+      <c r="K28" s="6" t="inlineStr">
+        <is>
+          <t>Valores del PR #62. El IEPS (8 %, base 22,22 y cuota 1,78) no es IVA. La base al 0 % no está impresa. El TC# largo no es el número del ticket.</t>
+        </is>
+      </c>
+    </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>

</xml_diff>